<commit_message>
feat: implement logic to force 'CONCLUÍDA' status for SEIs listed in `AUXILIAR.xlsx` and create a new file `0FF69500`.
</commit_message>
<xml_diff>
--- a/AUXILIAR.xlsx
+++ b/AUXILIAR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APRENDIZADO APP\MEDICOES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3CFC553-6EC1-4797-AC79-9404664903C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A75CB4-3EA3-4C69-83D5-A550DEC5B490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C423DC18-ADE7-4847-83C1-B9A17E509C00}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="365">
   <si>
     <t>NORTE</t>
   </si>
@@ -1109,6 +1109,33 @@
   </si>
   <si>
     <t>SOLVE CONSULTORIA E PROJETOS LTDA</t>
+  </si>
+  <si>
+    <t>170026/000821/2021</t>
+  </si>
+  <si>
+    <t>330018/001213/2022</t>
+  </si>
+  <si>
+    <t>330018/000569/2021</t>
+  </si>
+  <si>
+    <t>460001/000827/2023</t>
+  </si>
+  <si>
+    <t>460001/000821/2023</t>
+  </si>
+  <si>
+    <t>330018/001380/2022</t>
+  </si>
+  <si>
+    <t>330001/001441/2024</t>
+  </si>
+  <si>
+    <t>170026/001549/2020</t>
+  </si>
+  <si>
+    <t>330018/000567/2021</t>
   </si>
 </sst>
 </file>
@@ -1658,10 +1685,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{36ACF105-7C04-4C2F-BBBB-C0D7709C893E}" name="CONCLUIDAS" displayName="CONCLUIDAS" ref="M1:N20" totalsRowShown="0">
-  <autoFilter ref="M1:N20" xr:uid="{2C0FD495-D559-4428-9974-93B6DDD5F730}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M2:N20">
-    <sortCondition ref="M1:M20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{36ACF105-7C04-4C2F-BBBB-C0D7709C893E}" name="CONCLUIDAS" displayName="CONCLUIDAS" ref="M1:N29" totalsRowShown="0">
+  <autoFilter ref="M1:N29" xr:uid="{2C0FD495-D559-4428-9974-93B6DDD5F730}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M2:N22">
+    <sortCondition ref="M1:M22"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{BF27031E-8748-4BA6-8E8A-2457B029F7AB}" name="SEI" dataDxfId="1"/>
@@ -2077,8 +2104,8 @@
       <c r="K3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M3" s="11" t="s">
-        <v>21</v>
+      <c r="M3" s="14" t="s">
+        <v>356</v>
       </c>
       <c r="N3" s="12"/>
     </row>
@@ -2102,7 +2129,7 @@
         <v>27</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="N4" s="12"/>
     </row>
@@ -2126,7 +2153,7 @@
         <v>34</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="N5" s="12"/>
     </row>
@@ -2150,7 +2177,7 @@
         <v>41</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="N6" s="12"/>
     </row>
@@ -2174,7 +2201,7 @@
         <v>48</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="N7" s="12"/>
     </row>
@@ -2198,7 +2225,7 @@
         <v>55</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="N8" s="12"/>
     </row>
@@ -2222,7 +2249,7 @@
         <v>62</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="N9" s="12"/>
     </row>
@@ -2246,7 +2273,7 @@
         <v>69</v>
       </c>
       <c r="M10" s="11" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="N10" s="12"/>
     </row>
@@ -2270,7 +2297,7 @@
         <v>76</v>
       </c>
       <c r="M11" s="11" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="N11" s="12"/>
     </row>
@@ -2291,7 +2318,7 @@
         <v>82</v>
       </c>
       <c r="M12" s="11" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="N12" s="12"/>
     </row>
@@ -2312,7 +2339,7 @@
         <v>88</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="N13" s="12"/>
     </row>
@@ -2333,7 +2360,7 @@
         <v>94</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="N14" s="12"/>
     </row>
@@ -2354,7 +2381,7 @@
         <v>100</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="N15" s="12"/>
     </row>
@@ -2375,7 +2402,7 @@
         <v>354</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="N16" s="12"/>
     </row>
@@ -2393,7 +2420,7 @@
         <v>106</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="N17" s="12"/>
     </row>
@@ -2410,8 +2437,8 @@
       <c r="K18" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="M18" s="14" t="s">
-        <v>120</v>
+      <c r="M18" s="11" t="s">
+        <v>112</v>
       </c>
       <c r="N18" s="12"/>
     </row>
@@ -2428,8 +2455,8 @@
       <c r="K19" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="M19" s="15" t="s">
-        <v>125</v>
+      <c r="M19" s="14" t="s">
+        <v>120</v>
       </c>
       <c r="N19" s="12"/>
     </row>
@@ -2447,7 +2474,7 @@
         <v>347</v>
       </c>
       <c r="M20" s="15" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="N20" s="12"/>
     </row>
@@ -2464,6 +2491,10 @@
       <c r="K21" s="7" t="s">
         <v>116</v>
       </c>
+      <c r="M21" s="14" t="s">
+        <v>357</v>
+      </c>
+      <c r="N21" s="12"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B22" s="7" t="s">
@@ -2478,6 +2509,10 @@
       <c r="K22" s="7" t="s">
         <v>116</v>
       </c>
+      <c r="M22" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="N22" s="12"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B23" s="7" t="s">
@@ -2492,6 +2527,10 @@
       <c r="K23" s="7" t="s">
         <v>124</v>
       </c>
+      <c r="M23" s="14" t="s">
+        <v>358</v>
+      </c>
+      <c r="N23" s="12"/>
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" s="7" t="s">
@@ -2506,6 +2545,10 @@
       <c r="K24" s="7" t="s">
         <v>129</v>
       </c>
+      <c r="M24" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="N24" s="12"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B25" s="7" t="s">
@@ -2517,6 +2560,10 @@
       <c r="K25" s="7" t="s">
         <v>134</v>
       </c>
+      <c r="M25" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="N25" s="12"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B26" s="7" t="s">
@@ -2528,6 +2575,10 @@
       <c r="K26" s="7" t="s">
         <v>138</v>
       </c>
+      <c r="M26" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="N26" s="12"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="7" t="s">
@@ -2539,6 +2590,10 @@
       <c r="K27" s="7" t="s">
         <v>142</v>
       </c>
+      <c r="M27" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="N27" s="12"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B28" s="7" t="s">
@@ -2550,6 +2605,10 @@
       <c r="K28" s="7" t="s">
         <v>145</v>
       </c>
+      <c r="M28" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="N28" s="12"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B29" s="7" t="s">
@@ -2561,6 +2620,10 @@
       <c r="K29" s="7" t="s">
         <v>148</v>
       </c>
+      <c r="M29" s="14" t="s">
+        <v>364</v>
+      </c>
+      <c r="N29" s="12"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B30" s="7" t="s">

</xml_diff>

<commit_message>
fix: Corrected variable for assigning processed numeric cell values in `processa_medicoes.py`.
</commit_message>
<xml_diff>
--- a/AUXILIAR.xlsx
+++ b/AUXILIAR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APRENDIZADO APP\MEDICOES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A75CB4-3EA3-4C69-83D5-A550DEC5B490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65FF6631-26E6-4BD2-B4A0-DE10FAF4C298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C423DC18-ADE7-4847-83C1-B9A17E509C00}"/>
+    <workbookView xWindow="3720" yWindow="2520" windowWidth="21600" windowHeight="11295" xr2:uid="{C423DC18-ADE7-4847-83C1-B9A17E509C00}"/>
   </bookViews>
   <sheets>
     <sheet name="AUXILIAR" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="366">
   <si>
     <t>NORTE</t>
   </si>
@@ -1136,6 +1136,9 @@
   </si>
   <si>
     <t>330018/000567/2021</t>
+  </si>
+  <si>
+    <t>170026/000318/2022</t>
   </si>
 </sst>
 </file>
@@ -1685,8 +1688,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{36ACF105-7C04-4C2F-BBBB-C0D7709C893E}" name="CONCLUIDAS" displayName="CONCLUIDAS" ref="M1:N29" totalsRowShown="0">
-  <autoFilter ref="M1:N29" xr:uid="{2C0FD495-D559-4428-9974-93B6DDD5F730}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{36ACF105-7C04-4C2F-BBBB-C0D7709C893E}" name="CONCLUIDAS" displayName="CONCLUIDAS" ref="M1:N30" totalsRowShown="0">
+  <autoFilter ref="M1:N30" xr:uid="{2C0FD495-D559-4428-9974-93B6DDD5F730}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M2:N22">
     <sortCondition ref="M1:M22"/>
   </sortState>
@@ -2635,6 +2638,10 @@
       <c r="K30" s="7" t="s">
         <v>151</v>
       </c>
+      <c r="M30" s="14" t="s">
+        <v>365</v>
+      </c>
+      <c r="N30" s="12"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B31" s="7" t="s">

</xml_diff>

<commit_message>
Atualiza auxiliar e medicoes consolidadas
</commit_message>
<xml_diff>
--- a/AUXILIAR.xlsx
+++ b/AUXILIAR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APRENDIZADO APP\MEDICOES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A8C401D-E27C-426A-927C-E643C47EBB23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FBAFD2C-0D43-4505-8337-B8D06DE53678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C423DC18-ADE7-4847-83C1-B9A17E509C00}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="364">
   <si>
     <t>NORTE</t>
   </si>
@@ -1112,9 +1112,6 @@
   </si>
   <si>
     <t>170026/000821/2021</t>
-  </si>
-  <si>
-    <t>330018/001213/2022</t>
   </si>
   <si>
     <t>460001/000827/2023</t>
@@ -1685,10 +1682,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{36ACF105-7C04-4C2F-BBBB-C0D7709C893E}" name="CONCLUIDAS" displayName="CONCLUIDAS" ref="M1:N29" totalsRowShown="0">
-  <autoFilter ref="M1:N29" xr:uid="{2C0FD495-D559-4428-9974-93B6DDD5F730}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M2:N22">
-    <sortCondition ref="M1:M22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{36ACF105-7C04-4C2F-BBBB-C0D7709C893E}" name="CONCLUIDAS" displayName="CONCLUIDAS" ref="M1:N28" totalsRowShown="0">
+  <autoFilter ref="M1:N28" xr:uid="{2C0FD495-D559-4428-9974-93B6DDD5F730}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M2:N21">
+    <sortCondition ref="M1:M21"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{BF27031E-8748-4BA6-8E8A-2457B029F7AB}" name="SEI" dataDxfId="1"/>
@@ -2491,8 +2488,8 @@
       <c r="K21" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="M21" s="14" t="s">
-        <v>357</v>
+      <c r="M21" s="15" t="s">
+        <v>130</v>
       </c>
       <c r="N21" s="12"/>
     </row>
@@ -2509,8 +2506,8 @@
       <c r="K22" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="M22" s="15" t="s">
-        <v>130</v>
+      <c r="M22" s="14" t="s">
+        <v>357</v>
       </c>
       <c r="N22" s="12"/>
     </row>
@@ -2605,7 +2602,7 @@
       <c r="K28" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="M28" s="14" t="s">
+      <c r="M28" s="11" t="s">
         <v>363</v>
       </c>
       <c r="N28" s="12"/>
@@ -2620,10 +2617,6 @@
       <c r="K29" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="M29" s="11" t="s">
-        <v>364</v>
-      </c>
-      <c r="N29" s="12"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B30" s="7" t="s">

</xml_diff>